<commit_message>
Clean and consolidate Digital Resource Companion V1.0
</commit_message>
<xml_diff>
--- a/chapters/01/core/AIHE-A01/edit/xlsx/AIHE-A01_workbook.xlsx
+++ b/chapters/01/core/AIHE-A01/edit/xlsx/AIHE-A01_workbook.xlsx
@@ -180,12 +180,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="centre"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="centre"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -244,42 +244,42 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centre" vertical="centre" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>

</xml_diff>